<commit_message>
update production của từng phòng duoc bonus theo total stats
</commit_message>
<xml_diff>
--- a/docs/feature/economy-calculator-fixed.xlsx
+++ b/docs/feature/economy-calculator-fixed.xlsx
@@ -1,32 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hansentech-my.sharepoint.com/personal/davion_nguyen_hansencx_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WC\WORLDSCOLIDE\docs\feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="8_{B0F48902-DD4B-46E3-8B0F-E9C2C30808C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{484D9CE5-3F5B-4650-BF5B-D6626C4FE38B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224F6D04-9F3D-4AC3-A889-70A3099A4D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{126CF19B-DE03-4BC5-A902-1F108B4FCCAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{126CF19B-DE03-4BC5-A902-1F108B4FCCAA}"/>
   </bookViews>
   <sheets>
     <sheet name="economy-calculator-fixed" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="81">
-  <si>
-    <t>INPUT PARAMETERS</t>
-  </si>
-  <si>
-    <t>Difficulty Level</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="83">
   <si>
     <t>Easy</t>
   </si>
@@ -77,9 +82,6 @@
   </si>
   <si>
     <t>Members</t>
-  </si>
-  <si>
-    <t>Total Production</t>
   </si>
   <si>
     <t>Units</t>
@@ -264,13 +266,28 @@
   <si>
     <t>Ý Nghĩa của 0.8
 0.8 = Mỗi thành viên mới chỉ được 80% hiệu suất của thành viên trước đó</t>
+  </si>
+  <si>
+    <t>Scaling Factor</t>
+  </si>
+  <si>
+    <t>Total stats</t>
+  </si>
+  <si>
+    <t>Total Production before member stast</t>
+  </si>
+  <si>
+    <t>Member Stats Scaling Factor</t>
+  </si>
+  <si>
+    <t>Final production</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -407,6 +424,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -774,7 +797,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -787,6 +810,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1163,58 +1192,218 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5A4E69E-64D3-4E83-A84A-227AF999B9CD}">
-  <dimension ref="A5:J60"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="1" max="1" width="21.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" style="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="9.140625" style="1"/>
+    <col min="6" max="6" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="1"/>
     <col min="10" max="10" width="40.5703125" style="1" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="6">
+        <v>10</v>
+      </c>
+      <c r="C1" s="6">
+        <v>20</v>
+      </c>
+      <c r="D1" s="6">
+        <v>50</v>
+      </c>
+      <c r="E1" s="6">
+        <v>100</v>
+      </c>
+      <c r="F1" s="6">
+        <v>150</v>
+      </c>
+      <c r="G1" s="6">
+        <v>200</v>
+      </c>
+      <c r="H1" s="6">
+        <v>250</v>
+      </c>
+      <c r="I1" s="6">
+        <v>300</v>
+      </c>
+      <c r="J1" s="6">
+        <v>350</v>
+      </c>
+      <c r="K1" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="6">
+        <f xml:space="preserve"> 1 + 1.5 * (B1 / 400)</f>
+        <v>1.0375000000000001</v>
+      </c>
+      <c r="C2" s="6">
+        <f t="shared" ref="C2:K2" si="0" xml:space="preserve"> 1 + 1.5 * (C1 / 400)</f>
+        <v>1.075</v>
+      </c>
+      <c r="D2" s="6">
+        <f t="shared" si="0"/>
+        <v>1.1875</v>
+      </c>
+      <c r="E2" s="6">
+        <f t="shared" si="0"/>
+        <v>1.375</v>
+      </c>
+      <c r="F2" s="6">
+        <f t="shared" si="0"/>
+        <v>1.5625</v>
+      </c>
+      <c r="G2" s="6">
+        <f t="shared" si="0"/>
+        <v>1.75</v>
+      </c>
+      <c r="H2" s="6">
+        <f t="shared" si="0"/>
+        <v>1.9375</v>
+      </c>
+      <c r="I2" s="6">
+        <f t="shared" si="0"/>
+        <v>2.125</v>
+      </c>
+      <c r="J2" s="6">
+        <f t="shared" si="0"/>
+        <v>2.3125</v>
+      </c>
+      <c r="K2" s="6">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="E5" s="4">
+        <v>3.375</v>
+      </c>
+      <c r="F5" s="4">
+        <v>5.0625</v>
+      </c>
+      <c r="G5" s="4">
+        <v>7.59375</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="E6" s="4">
+        <v>3.375</v>
+      </c>
+      <c r="F6" s="4">
+        <v>5.0625</v>
+      </c>
+      <c r="G6" s="4">
+        <v>7.59375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="E7" s="4">
+        <v>3.375</v>
+      </c>
+      <c r="F7" s="4">
+        <v>5.0625</v>
+      </c>
+      <c r="G7" s="4">
+        <v>7.59375</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="E8" s="4">
+        <v>3.375</v>
+      </c>
+      <c r="F8" s="4">
+        <v>5.0625</v>
+      </c>
+      <c r="G8" s="4">
+        <v>7.59375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B9" s="4">
         <v>1</v>
@@ -1235,436 +1424,433 @@
         <v>7.59375</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="4">
-        <v>1</v>
-      </c>
-      <c r="C10" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="D10" s="4">
-        <v>2.25</v>
-      </c>
-      <c r="E10" s="4">
-        <v>3.375</v>
-      </c>
-      <c r="F10" s="4">
-        <v>5.0625</v>
-      </c>
-      <c r="G10" s="4">
-        <v>7.59375</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="4">
         <v>1</v>
       </c>
       <c r="C11" s="4">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D11" s="4">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="E11" s="4">
-        <v>3.375</v>
+        <v>4</v>
       </c>
       <c r="F11" s="4">
-        <v>5.0625</v>
+        <v>5</v>
       </c>
       <c r="G11" s="4">
-        <v>7.59375</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="H11" s="4">
+        <v>7</v>
+      </c>
+      <c r="I11" s="4">
+        <v>8</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>7</v>
+        <v>72</v>
       </c>
       <c r="B12" s="4">
-        <v>1</v>
+        <f>(0.25*(0.8)^(1-1))</f>
+        <v>0.25</v>
       </c>
       <c r="C12" s="4">
-        <v>1.5</v>
+        <f>(0.25*(0.8)^(2-1))</f>
+        <v>0.2</v>
       </c>
       <c r="D12" s="4">
-        <v>2.25</v>
+        <f>(0.25*(0.8)^(3-1))</f>
+        <v>0.16000000000000003</v>
       </c>
       <c r="E12" s="4">
-        <v>3.375</v>
+        <f>(0.25*(0.8)^(4-1))</f>
+        <v>0.12800000000000003</v>
       </c>
       <c r="F12" s="4">
-        <v>5.0625</v>
+        <f>(0.25*(0.8)^(5-1))</f>
+        <v>0.10240000000000005</v>
       </c>
       <c r="G12" s="4">
-        <v>7.59375</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <f>(0.25*(0.8)^(6-1))</f>
+        <v>8.1920000000000048E-2</v>
+      </c>
+      <c r="H12" s="4">
+        <f>(0.25*(0.8)^(7-1))</f>
+        <v>6.5536000000000039E-2</v>
+      </c>
+      <c r="I12" s="4">
+        <f>(0.25*(0.8)^(8-1))</f>
+        <v>5.2428800000000039E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="4">
-        <v>1</v>
+        <f>B12</f>
+        <v>0.25</v>
       </c>
       <c r="C13" s="4">
-        <v>1.5</v>
+        <f>B12+C12</f>
+        <v>0.45</v>
       </c>
       <c r="D13" s="4">
-        <v>2.25</v>
+        <f>C13+D12</f>
+        <v>0.6100000000000001</v>
       </c>
       <c r="E13" s="4">
-        <v>3.375</v>
+        <f t="shared" ref="E13:I13" si="1">D13+E12</f>
+        <v>0.7380000000000001</v>
       </c>
       <c r="F13" s="4">
-        <v>5.0625</v>
+        <f t="shared" si="1"/>
+        <v>0.84040000000000015</v>
       </c>
       <c r="G13" s="4">
-        <v>7.59375</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0.92232000000000025</v>
+      </c>
+      <c r="H13" s="4">
+        <f t="shared" si="1"/>
+        <v>0.98785600000000029</v>
+      </c>
+      <c r="I13" s="4">
+        <f t="shared" si="1"/>
+        <v>1.0402848000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="4">
+        <f>B12</f>
+        <v>0.25</v>
+      </c>
+      <c r="C14" s="4">
+        <f>B12+C12</f>
+        <v>0.45</v>
+      </c>
+      <c r="D14" s="4">
+        <f>C14+D12</f>
+        <v>0.6100000000000001</v>
+      </c>
+      <c r="E14" s="4">
+        <f t="shared" ref="E14:I14" si="2">D14+E12</f>
+        <v>0.7380000000000001</v>
+      </c>
+      <c r="F14" s="4">
+        <f t="shared" si="2"/>
+        <v>0.84040000000000015</v>
+      </c>
+      <c r="G14" s="4">
+        <f t="shared" si="2"/>
+        <v>0.92232000000000025</v>
+      </c>
+      <c r="H14" s="4">
+        <f t="shared" si="2"/>
+        <v>0.98785600000000029</v>
+      </c>
+      <c r="I14" s="4">
+        <f t="shared" si="2"/>
+        <v>1.0402848000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" s="4">
-        <v>1</v>
+        <f>B12</f>
+        <v>0.25</v>
       </c>
       <c r="C15" s="4">
-        <v>2</v>
+        <f>B12+C12</f>
+        <v>0.45</v>
       </c>
       <c r="D15" s="4">
-        <v>3</v>
+        <f>C15+D12</f>
+        <v>0.6100000000000001</v>
       </c>
       <c r="E15" s="4">
-        <v>4</v>
+        <f t="shared" ref="E15:I15" si="3">D15+E12</f>
+        <v>0.7380000000000001</v>
       </c>
       <c r="F15" s="4">
-        <v>5</v>
+        <f t="shared" si="3"/>
+        <v>0.84040000000000015</v>
       </c>
       <c r="G15" s="4">
-        <v>6</v>
+        <f t="shared" si="3"/>
+        <v>0.92232000000000025</v>
       </c>
       <c r="H15" s="4">
-        <v>7</v>
+        <f t="shared" si="3"/>
+        <v>0.98785600000000029</v>
       </c>
       <c r="I15" s="4">
-        <v>8</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" s="4">
-        <f>(0.25*(0.8)^(1-1))</f>
-        <v>0.25</v>
-      </c>
-      <c r="C16" s="4">
-        <f>(0.25*(0.8)^(2-1))</f>
-        <v>0.2</v>
-      </c>
-      <c r="D16" s="4">
-        <f>(0.25*(0.8)^(3-1))</f>
-        <v>0.16000000000000003</v>
-      </c>
-      <c r="E16" s="4">
-        <f>(0.25*(0.8)^(4-1))</f>
-        <v>0.12800000000000003</v>
-      </c>
-      <c r="F16" s="4">
-        <f>(0.25*(0.8)^(5-1))</f>
-        <v>0.10240000000000005</v>
-      </c>
-      <c r="G16" s="4">
-        <f>(0.25*(0.8)^(6-1))</f>
-        <v>8.1920000000000048E-2</v>
-      </c>
-      <c r="H16" s="4">
-        <f>(0.25*(0.8)^(7-1))</f>
-        <v>6.5536000000000039E-2</v>
-      </c>
-      <c r="I16" s="4">
-        <f>(0.25*(0.8)^(8-1))</f>
-        <v>5.2428800000000039E-2</v>
+        <f t="shared" si="3"/>
+        <v>1.0402848000000002</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="4">
-        <f>B16</f>
-        <v>0.25</v>
-      </c>
-      <c r="C17" s="4">
-        <f>B16+C16</f>
-        <v>0.45</v>
-      </c>
-      <c r="D17" s="4">
-        <f>C17+D16</f>
-        <v>0.6100000000000001</v>
-      </c>
-      <c r="E17" s="4">
-        <f t="shared" ref="E17:I17" si="0">D17+E16</f>
-        <v>0.7380000000000001</v>
-      </c>
-      <c r="F17" s="4">
-        <f t="shared" si="0"/>
-        <v>0.84040000000000015</v>
-      </c>
-      <c r="G17" s="4">
-        <f t="shared" si="0"/>
-        <v>0.92232000000000025</v>
-      </c>
-      <c r="H17" s="4">
-        <f t="shared" si="0"/>
-        <v>0.98785600000000029</v>
-      </c>
-      <c r="I17" s="4">
-        <f t="shared" si="0"/>
-        <v>1.0402848000000002</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" s="4">
-        <f>B16</f>
-        <v>0.25</v>
-      </c>
-      <c r="C18" s="4">
-        <f>B16+C16</f>
-        <v>0.45</v>
-      </c>
-      <c r="D18" s="4">
-        <f>C18+D16</f>
-        <v>0.6100000000000001</v>
-      </c>
-      <c r="E18" s="4">
-        <f t="shared" ref="E18:I18" si="1">D18+E16</f>
-        <v>0.7380000000000001</v>
-      </c>
-      <c r="F18" s="4">
-        <f t="shared" si="1"/>
-        <v>0.84040000000000015</v>
-      </c>
-      <c r="G18" s="4">
-        <f t="shared" si="1"/>
-        <v>0.92232000000000025</v>
-      </c>
-      <c r="H18" s="4">
-        <f t="shared" si="1"/>
-        <v>0.98785600000000029</v>
-      </c>
-      <c r="I18" s="4">
-        <f t="shared" si="1"/>
-        <v>1.0402848000000002</v>
+        <v>12</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B19" s="4">
-        <f>B16</f>
-        <v>0.25</v>
+        <v>10</v>
       </c>
       <c r="C19" s="4">
-        <f>B16+C16</f>
-        <v>0.45</v>
+        <f>G5</f>
+        <v>7.59375</v>
       </c>
       <c r="D19" s="4">
-        <f>C19+D16</f>
-        <v>0.6100000000000001</v>
+        <f>C19*B19</f>
+        <v>75.9375</v>
       </c>
       <c r="E19" s="4">
-        <f t="shared" ref="E19:I19" si="2">D19+E16</f>
-        <v>0.7380000000000001</v>
+        <f>I13</f>
+        <v>1.0402848000000002</v>
       </c>
       <c r="F19" s="4">
-        <f t="shared" si="2"/>
-        <v>0.84040000000000015</v>
+        <f>D19*(1+E19)</f>
+        <v>154.93412700000002</v>
       </c>
       <c r="G19" s="4">
-        <f t="shared" si="2"/>
-        <v>0.92232000000000025</v>
+        <v>2.5</v>
       </c>
       <c r="H19" s="4">
-        <f t="shared" si="2"/>
-        <v>0.98785600000000029</v>
-      </c>
-      <c r="I19" s="4">
-        <f t="shared" si="2"/>
+        <f>F19*G19</f>
+        <v>387.33531750000003</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>8</v>
+      </c>
+      <c r="C20" s="4">
+        <f t="shared" ref="C20:C21" si="4">G6</f>
+        <v>7.59375</v>
+      </c>
+      <c r="D20" s="4">
+        <f t="shared" ref="D20:D21" si="5">C20*B20</f>
+        <v>60.75</v>
+      </c>
+      <c r="E20" s="4">
+        <f t="shared" ref="E20:E21" si="6">I14</f>
         <v>1.0402848000000002</v>
+      </c>
+      <c r="F20" s="4">
+        <f t="shared" ref="F20:F21" si="7">D20*(1+E20)</f>
+        <v>123.94730160000002</v>
+      </c>
+      <c r="G20" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="H20" s="4">
+        <f t="shared" ref="H20:H21" si="8">F20*G20</f>
+        <v>309.86825400000004</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4">
+        <v>6</v>
+      </c>
+      <c r="C21" s="4">
+        <f t="shared" si="4"/>
+        <v>7.59375</v>
+      </c>
+      <c r="D21" s="4">
+        <f t="shared" si="5"/>
+        <v>45.5625</v>
+      </c>
+      <c r="E21" s="4">
+        <f t="shared" si="6"/>
+        <v>1.0402848000000002</v>
+      </c>
+      <c r="F21" s="4">
+        <f t="shared" si="7"/>
+        <v>92.960476200000016</v>
+      </c>
+      <c r="G21" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="H21" s="4">
+        <f t="shared" si="8"/>
+        <v>232.40119050000004</v>
+      </c>
+      <c r="I21" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="4">
-        <v>10</v>
-      </c>
-      <c r="C23" s="4">
-        <f>G9</f>
-        <v>7.59375</v>
-      </c>
-      <c r="D23" s="4">
-        <f>C23*B23</f>
-        <v>75.9375</v>
-      </c>
-      <c r="E23" s="4">
-        <f>I17</f>
-        <v>1.0402848000000002</v>
-      </c>
-      <c r="F23" s="4">
-        <f>D23*(1+E23)</f>
-        <v>154.93412700000002</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="4">
-        <v>8</v>
-      </c>
-      <c r="C24" s="4">
-        <f t="shared" ref="C24:C25" si="3">G10</f>
-        <v>7.59375</v>
-      </c>
-      <c r="D24" s="4">
-        <f t="shared" ref="D24:D25" si="4">C24*B24</f>
-        <v>60.75</v>
-      </c>
-      <c r="E24" s="4">
-        <f t="shared" ref="E24:E25" si="5">I18</f>
-        <v>1.0402848000000002</v>
-      </c>
-      <c r="F24" s="4">
-        <f t="shared" ref="F24:F25" si="6">D24*(1+E24)</f>
-        <v>123.94730160000002</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>78</v>
+      <c r="B24" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" s="4">
-        <v>6</v>
-      </c>
-      <c r="C25" s="4">
-        <f t="shared" si="3"/>
-        <v>7.59375</v>
-      </c>
-      <c r="D25" s="4">
-        <f t="shared" si="4"/>
-        <v>45.5625</v>
-      </c>
-      <c r="E25" s="4">
-        <f t="shared" si="5"/>
-        <v>1.0402848000000002</v>
-      </c>
-      <c r="F25" s="4">
-        <f t="shared" si="6"/>
-        <v>92.960476200000016</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>79</v>
+      <c r="A25" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="3">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="C25" s="1" t="e">
+        <f>F18*B24</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D25" s="1" t="e">
+        <f>F18*B24*0.3</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E25" s="1" t="e">
+        <f>F18*B24*0.1</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="C26" s="1" t="e">
+        <f>F18*B25</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D26" s="1" t="e">
+        <f>F18*B25*0.3</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E26" s="1" t="e">
+        <f>F18*B25*0.1</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
+      </c>
+      <c r="B27" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="C27" s="1" t="e">
+        <f>F18*B25</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D27" s="1" t="e">
+        <f>F18*B25*0.3</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E27" s="1" t="e">
+        <f>F18*B25*0.1</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="3">
-        <v>6.5000000000000002E-2</v>
-      </c>
-      <c r="C29" s="1" t="e">
-        <f>F22*B28</f>
+      <c r="B28" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="C28" s="1" t="e">
+        <f>F18*B25</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D29" s="1" t="e">
-        <f>F22*B28*0.3</f>
+      <c r="D28" s="1" t="e">
+        <f>F18*B25*0.3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E29" s="1" t="e">
-        <f>F22*B28*0.1</f>
+      <c r="E28" s="1" t="e">
+        <f>F18*B25*0.1</f>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -1672,424 +1858,364 @@
       <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="3">
-        <v>0.125</v>
-      </c>
-      <c r="C30" s="1" t="e">
-        <f>F22*B29</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D30" s="1" t="e">
-        <f>F22*B29*0.3</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E30" s="1" t="e">
-        <f>F22*B29*0.1</f>
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="3">
-        <v>0.125</v>
-      </c>
-      <c r="C31" s="1" t="e">
-        <f>F22*B29</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D31" s="1" t="e">
-        <f>F22*B29*0.3</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E31" s="1" t="e">
-        <f>F22*B29*0.1</f>
-        <v>#VALUE!</v>
+      <c r="C31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0</v>
+      </c>
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="3">
-        <v>0.125</v>
-      </c>
-      <c r="C32" s="1" t="e">
-        <f>F22*B29</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D32" s="1" t="e">
-        <f>F22*B29*0.3</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E32" s="1" t="e">
-        <f>F22*B29*0.1</f>
-        <v>#VALUE!</v>
+      <c r="B33" s="1">
+        <v>11.5</v>
+      </c>
+      <c r="C33" s="1">
+        <v>9</v>
+      </c>
+      <c r="D33" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
+      </c>
+      <c r="B34" s="1">
+        <v>113.67</v>
+      </c>
+      <c r="C34" s="1">
+        <v>12</v>
+      </c>
+      <c r="D34" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D35" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="1">
         <v>21</v>
+      </c>
+      <c r="C35" s="1">
+        <v>13.5</v>
+      </c>
+      <c r="D35" s="1">
+        <v>9</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="B36" s="1">
-        <v>0.33</v>
+        <v>35</v>
       </c>
       <c r="C36" s="1">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D36" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37" s="1">
-        <v>11.5</v>
-      </c>
-      <c r="C37" s="1">
-        <v>9</v>
-      </c>
-      <c r="D37" s="1">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="1">
-        <v>113.67</v>
-      </c>
-      <c r="C38" s="1">
-        <v>12</v>
-      </c>
-      <c r="D38" s="1">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B39" s="1">
-        <v>21</v>
-      </c>
-      <c r="C39" s="1">
-        <v>13.5</v>
-      </c>
-      <c r="D39" s="1">
-        <v>9</v>
+        <v>12</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B40" s="1">
-        <v>35</v>
-      </c>
-      <c r="C40" s="1">
-        <v>15</v>
-      </c>
-      <c r="D40" s="1">
-        <v>15</v>
+        <v>24</v>
+      </c>
+      <c r="B40" s="1" t="e">
+        <f>C26</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C40" s="1" t="e">
+        <f>VLOOKUP(#REF!,B32:D36,2,FALSE)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="D40" s="1" t="e">
+        <f>B39-C39</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E40" s="1" t="str">
+        <f>IF(D39&gt;0,"SURPLUS","DEFICIT")</f>
+        <v>SURPLUS</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="1" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C41" s="1" t="e">
+        <f>VLOOKUP(#REF!,B32:D36,3,FALSE)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="D41" s="1" t="e">
+        <f>B40-C40</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E41" s="1" t="e">
+        <f>IF(D40&gt;0,"SURPLUS","DEFICIT")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>41</v>
+        <v>18</v>
+      </c>
+      <c r="B42" s="1">
+        <f>F17</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="1" t="e">
+        <f>VLOOKUP(#REF!,B32:D36,4,FALSE)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="D42" s="1" t="e">
+        <f>B41-C41</f>
+        <v>#REF!</v>
+      </c>
+      <c r="E42" s="1" t="e">
+        <f>IF(D41&gt;0,"SURPLUS","DEFICIT")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B44" s="1" t="e">
-        <f>C30</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C44" s="1" t="e">
-        <f>VLOOKUP(B6,B36:D40,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D44" s="1" t="e">
-        <f>B43-C43</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E44" s="1" t="str">
-        <f>IF(D43&gt;0,"SURPLUS","DEFICIT")</f>
-        <v>SURPLUS</v>
+        <v>39</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B45" s="1" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C45" s="1" t="e">
-        <f>VLOOKUP(B6,B36:D40,3,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D45" s="1" t="e">
-        <f>B44-C44</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E45" s="1" t="e">
-        <f>IF(D44&gt;0,"SURPLUS","DEFICIT")</f>
-        <v>#VALUE!</v>
+        <v>40</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B46" s="1">
-        <f>F21</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="1" t="e">
-        <f>VLOOKUP(B6,B36:D40,4,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D46" s="1" t="e">
-        <f>B45-C45</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E46" s="1" t="e">
-        <f>IF(D45&gt;0,"SURPLUS","DEFICIT")</f>
-        <v>#VALUE!</v>
+        <v>44</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
+      </c>
+      <c r="B52" s="1">
+        <v>0</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0</v>
+      </c>
+      <c r="E52" s="1">
+        <v>9</v>
+      </c>
+      <c r="F52" s="1" t="e">
+        <f>SUM(D39:D41)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" s="1">
+        <v>2</v>
+      </c>
+      <c r="C53" s="1">
+        <v>2</v>
+      </c>
+      <c r="D53" s="1">
+        <v>2</v>
+      </c>
+      <c r="E53" s="1">
+        <v>9</v>
+      </c>
+      <c r="F53" s="1" t="e">
+        <f>SUM(D39:D41)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
+      </c>
+      <c r="B54" s="1">
+        <v>1</v>
+      </c>
+      <c r="C54" s="1">
+        <v>3</v>
+      </c>
+      <c r="D54" s="1">
+        <v>0</v>
+      </c>
+      <c r="E54" s="1">
+        <v>9</v>
+      </c>
+      <c r="F54" s="1" t="e">
+        <f>SUM(D39:D41)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+      <c r="B55" s="1">
+        <v>1</v>
+      </c>
+      <c r="C55" s="1">
+        <v>0</v>
+      </c>
+      <c r="D55" s="1">
+        <v>3</v>
+      </c>
+      <c r="E55" s="1">
+        <v>9</v>
+      </c>
+      <c r="F55" s="1" t="e">
+        <f>SUM(D39:D41)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B56" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C56" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D56" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E56" s="1">
         <v>9</v>
       </c>
       <c r="F56" s="1" t="e">
-        <f>SUM(D43:D45)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B57" s="1">
-        <v>2</v>
-      </c>
-      <c r="C57" s="1">
-        <v>2</v>
-      </c>
-      <c r="D57" s="1">
-        <v>2</v>
-      </c>
-      <c r="E57" s="1">
-        <v>9</v>
-      </c>
-      <c r="F57" s="1" t="e">
-        <f>SUM(D43:D45)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B58" s="1">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1">
-        <v>3</v>
-      </c>
-      <c r="D58" s="1">
-        <v>0</v>
-      </c>
-      <c r="E58" s="1">
-        <v>9</v>
-      </c>
-      <c r="F58" s="1" t="e">
-        <f>SUM(D43:D45)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B59" s="1">
-        <v>1</v>
-      </c>
-      <c r="C59" s="1">
-        <v>0</v>
-      </c>
-      <c r="D59" s="1">
-        <v>3</v>
-      </c>
-      <c r="E59" s="1">
-        <v>9</v>
-      </c>
-      <c r="F59" s="1" t="e">
-        <f>SUM(D43:D45)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B60" s="1">
-        <v>5</v>
-      </c>
-      <c r="C60" s="1">
-        <v>5</v>
-      </c>
-      <c r="D60" s="1">
-        <v>5</v>
-      </c>
-      <c r="E60" s="1">
-        <v>9</v>
-      </c>
-      <c r="F60" s="1" t="e">
-        <f>SUM(D43:D45)</f>
+        <f>SUM(D39:D41)</f>
         <v>#VALUE!</v>
       </c>
     </row>

</xml_diff>